<commit_message>
Added: Sample Email in the Candidate Excel sheet
</commit_message>
<xml_diff>
--- a/Data/Input/CandidateInfo.xlsx
+++ b/Data/Input/CandidateInfo.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UiPathProjects\HR_GENERATE_OFFER_LETTER_FILES\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://claysysmail-my.sharepoint.com/personal/manish_unnikrishnan_claysys_net/Documents/Documents/UiPath/Dispatcher-HR_Offer_Letter_Generation/Data/Input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E3C2486-8807-4759-BDE9-97585A1CEF06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="13_ncr:1_{8E3C2486-8807-4759-BDE9-97585A1CEF06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B6F9D3FE-409F-4734-A1E1-F769310859BF}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{57A7E307-140A-483A-BD81-E14EABD2E01B}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="60">
   <si>
     <t>Date</t>
   </si>
@@ -202,16 +202,19 @@
     <t>Loreta</t>
   </si>
   <si>
-    <t>mukeshkala@outlook.com</t>
-  </si>
-  <si>
-    <t>mukeshkalaoutlook.co</t>
-  </si>
-  <si>
-    <t>mukeoutlook.com</t>
-  </si>
-  <si>
     <t>Sno</t>
+  </si>
+  <si>
+    <t>manishappu678@gmail.com</t>
+  </si>
+  <si>
+    <t>manishappu789@gmail.com</t>
+  </si>
+  <si>
+    <t>manishappu789@gmail.co</t>
+  </si>
+  <si>
+    <t>manish@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -255,7 +258,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -285,17 +288,6 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
       <top style="thin">
         <color indexed="64"/>
       </top>
@@ -307,7 +299,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
@@ -318,9 +310,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -650,7 +640,7 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B1" s="6" t="s">
         <v>2</v>
@@ -664,13 +654,13 @@
       <c r="E1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="F1" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="G1" s="8" t="s">
+      <c r="G1" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="7" t="s">
+      <c r="H1" s="6" t="s">
         <v>35</v>
       </c>
     </row>
@@ -696,8 +686,8 @@
       <c r="G2" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="H2" s="9" t="s">
-        <v>55</v>
+      <c r="H2" s="8" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -722,8 +712,8 @@
       <c r="G3" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="H3" s="9" t="s">
-        <v>55</v>
+      <c r="H3" s="8" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -748,8 +738,8 @@
       <c r="G4" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="H4" s="9" t="s">
-        <v>55</v>
+      <c r="H4" s="8" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -774,8 +764,8 @@
       <c r="G5" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="H5" s="9" t="s">
-        <v>55</v>
+      <c r="H5" s="8" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -800,8 +790,8 @@
       <c r="G6" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="H6" s="9" t="s">
-        <v>55</v>
+      <c r="H6" s="8" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -826,8 +816,8 @@
       <c r="G7" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="H7" s="10" t="s">
-        <v>55</v>
+      <c r="H7" s="8" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -852,8 +842,8 @@
       <c r="G8" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="H8" s="9" t="s">
-        <v>55</v>
+      <c r="H8" s="8" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -878,8 +868,8 @@
       <c r="G9" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="H9" s="9" t="s">
-        <v>55</v>
+      <c r="H9" s="8" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -904,8 +894,8 @@
       <c r="G10" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="H10" s="10" t="s">
-        <v>56</v>
+      <c r="H10" s="8" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -930,8 +920,8 @@
       <c r="G11" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="H11" s="9" t="s">
-        <v>55</v>
+      <c r="H11" s="8" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -956,8 +946,8 @@
       <c r="G12" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="H12" s="9" t="s">
-        <v>55</v>
+      <c r="H12" s="8" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -982,8 +972,8 @@
       <c r="G13" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="H13" s="9" t="s">
-        <v>55</v>
+      <c r="H13" s="8" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
@@ -1008,8 +998,8 @@
       <c r="G14" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="H14" s="9" t="s">
-        <v>55</v>
+      <c r="H14" s="8" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
@@ -1034,7 +1024,7 @@
       <c r="G15" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="H15" s="9"/>
+      <c r="H15" s="8"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
@@ -1058,8 +1048,8 @@
       <c r="G16" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="H16" s="9" t="s">
-        <v>55</v>
+      <c r="H16" s="8" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
@@ -1084,8 +1074,8 @@
       <c r="G17" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="H17" s="9" t="s">
-        <v>55</v>
+      <c r="H17" s="8" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
@@ -1110,8 +1100,8 @@
       <c r="G18" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="H18" s="9" t="s">
-        <v>57</v>
+      <c r="H18" s="8" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
@@ -1136,8 +1126,8 @@
       <c r="G19" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="H19" s="9" t="s">
-        <v>55</v>
+      <c r="H19" s="8" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
@@ -1162,8 +1152,8 @@
       <c r="G20" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="H20" s="9" t="s">
-        <v>55</v>
+      <c r="H20" s="8" t="s">
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>